<commit_message>
Hata Kayitlari tek sayfaya sigsin (Excel baslik tekrarini uygulamiyor)
Kurum Excel kullaniyor; formu bu makinedeki Excel 2010'da acip kendi PDF
ciktisini aldim. Onceki committe ikinci sayfaya tasan kayitlar icin
konulan baslik tekrari (print_title_rows) LibreOffice'te calisiyor ama
EXCEL'DE CALISMIYOR: PageSetup.PrintTitleRows bos donuyor ve Excel'in
kendi API'siyle kurulup kaydedildiginde bile cikti basliksiz kaliyor
(ustelik dosya adindan turetilmis bozuk bir tanimli ad uretiyor).

Mekanizmayla ugrasmak yerine sorunu kaldirdim: sayfa tek sayfaya
sigdiriliyor (fitToHeight), boylece ikinci sayfa hic olusmuyor ve
12 kaydin tamami basligiyla birlikte tek yatay A4'te duruyor.

Excel ciktisiyla dogrulandi: 8 sayfa, hepsi tam A4, Ogrenci/Ogretmen
sayfa sonlari bolum sinirinda, formul calisiyor.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ortaokul/SeFu_Ortaokul_Pilot_Geri_Bildirim_Formu.xlsx
+++ b/ortaokul/SeFu_Ortaokul_Pilot_Geri_Bildirim_Formu.xlsx
@@ -15,9 +15,6 @@
     <sheet name="Hata Kayıtları" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Hafta Sonu" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
-  <definedNames>
-    <definedName function="false" hidden="false" localSheetId="4" name="_xlnm.Print_Titles" vbProcedure="false">'Hata Kayıtları'!$3:$3</definedName>
-  </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -1811,7 +1808,7 @@
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.5" right="0.4" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>